<commit_message>
Add requirements.txt and fix netlify.toml for Python deps
</commit_message>
<xml_diff>
--- a/雅各組出席表.xlsx
+++ b/雅各組出席表.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="25">
   <si>
     <t>序號</t>
   </si>
@@ -583,7 +583,7 @@
       </c>
     </row>
     <row r="2" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="3" spans="1:5" ht="79.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -684,10 +684,14 @@
       <c r="B9" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
+      <c r="C9" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>22</v>
+      </c>
       <c r="E9" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -802,7 +806,9 @@
       <c r="B17" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C17" s="3"/>
+      <c r="C17" s="3" t="s">
+        <v>22</v>
+      </c>
       <c r="D17" s="3"/>
       <c r="E17" s="3" t="s">
         <v>23</v>
@@ -815,7 +821,9 @@
       <c r="B18" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C18" s="3"/>
+      <c r="C18" s="3" t="s">
+        <v>22</v>
+      </c>
       <c r="D18" s="3"/>
       <c r="E18" s="3" t="s">
         <v>23</v>
@@ -832,5 +840,6 @@
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>